<commit_message>
Updated according to announcement on brightspace
</commit_message>
<xml_diff>
--- a/xlsx/hw3.xlsx
+++ b/xlsx/hw3.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\81303\source\repos\JasperPQ\xll_ml\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xll_ml-master\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A65F775-AE32-48C1-9430-9C48F64BC9B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{479B3633-4C3D-4984-9860-87561442E57B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6690" yWindow="1395" windowWidth="21600" windowHeight="11835" xr2:uid="{EA092A42-1670-4D44-86F1-B9E7694F8A62}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>f</t>
   </si>
@@ -79,6 +79,22 @@
   </si>
   <si>
     <t>m</t>
+  </si>
+  <si>
+    <t>k</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>moneyness</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>call</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>put</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -547,14 +563,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE06CDEE-4F3C-473F-9F8B-5F0D6CBFE894}">
-  <dimension ref="B3:C7"/>
+  <dimension ref="B3:G17"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="3.59765625" customWidth="1"/>
     <col min="3" max="3" width="11.69921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.09765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3">
+    <row r="3" spans="2:7">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -562,7 +579,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="2:3">
+    <row r="4" spans="2:7">
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
@@ -570,7 +587,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="5" spans="2:3">
+    <row r="5" spans="2:7">
       <c r="B5" s="1" t="s">
         <v>2</v>
       </c>
@@ -578,22 +595,166 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="2:3">
+    <row r="6" spans="2:7">
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="2" cm="1">
         <f t="array" ref="C6">_xll.\OPTION.NORMAL()</f>
-        <v>2410180663760</v>
-      </c>
-    </row>
-    <row r="7" spans="2:3">
+        <v>2859249174912</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C7" s="3" cm="1">
         <f t="array" ref="C7">_xll.OPTION.BLACK.PUT(f, s, k, m)</f>
         <v>3.9877746125013118</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7">
+      <c r="D8" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7">
+      <c r="D9" cm="1">
+        <f t="array" ref="D9:D17">_xlfn.SEQUENCE(9, 1, 80, 5)</f>
+        <v>80</v>
+      </c>
+      <c r="E9" cm="1">
+        <f t="array" ref="E9:E17">_xlfn.MAP(_xlfn.ANCHORARRAY(D9),_xlfn.LAMBDA(_xlpm.k,_xll.OPTION.BLACK.MONEYNESS(f,s,_xlpm.k,m)))</f>
+        <v>-2.1814355131420968</v>
+      </c>
+      <c r="F9" cm="1">
+        <f t="array" ref="F9:F17">_xlfn.MAP(_xlfn.ANCHORARRAY(D9),_xlfn.LAMBDA(_xlpm.k,_xll.OPTION.BLACK.CALL(f,s,_xlpm.k,m)))</f>
+        <v>20.039913489502155</v>
+      </c>
+      <c r="G9" cm="1">
+        <f t="array" ref="G9:G17">_xlfn.MAP(_xlfn.ANCHORARRAY(D9),_xlfn.LAMBDA(_xlpm.k,_xll.OPTION.BLACK.PUT(f,s,_xlpm.k,m)))</f>
+        <v>3.9913489502149124E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7">
+      <c r="D10">
+        <v>85</v>
+      </c>
+      <c r="E10">
+        <v>-1.5751892949777493</v>
+      </c>
+      <c r="F10">
+        <v>15.201690203245803</v>
+      </c>
+      <c r="G10">
+        <v>0.20169020324580078</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7">
+      <c r="D11">
+        <v>90</v>
+      </c>
+      <c r="E11">
+        <v>-1.0036051565782627</v>
+      </c>
+      <c r="F11">
+        <v>10.71237738374009</v>
+      </c>
+      <c r="G11">
+        <v>0.7123773837400833</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7">
+      <c r="D12">
+        <v>95</v>
+      </c>
+      <c r="E12">
+        <v>-0.46293294387550571</v>
+      </c>
+      <c r="F12">
+        <v>6.8880683097281832</v>
+      </c>
+      <c r="G12">
+        <v>1.8880683097281832</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7">
+      <c r="D13">
+        <v>100</v>
+      </c>
+      <c r="E13">
+        <v>5.000000000000001E-2</v>
+      </c>
+      <c r="F13">
+        <v>3.9877746125013118</v>
+      </c>
+      <c r="G13">
+        <v>3.9877746125013118</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7">
+      <c r="D14">
+        <v>105</v>
+      </c>
+      <c r="E14">
+        <v>0.53790164169432031</v>
+      </c>
+      <c r="F14">
+        <v>2.0640245213143373</v>
+      </c>
+      <c r="G14">
+        <v>7.0640245213143373</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7">
+      <c r="D15">
+        <v>110</v>
+      </c>
+      <c r="E15">
+        <v>1.0031017980432493</v>
+      </c>
+      <c r="F15">
+        <v>0.95394336557325232</v>
+      </c>
+      <c r="G15">
+        <v>10.953943365573252</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7">
+      <c r="D16">
+        <v>115</v>
+      </c>
+      <c r="E16">
+        <v>1.4476194237515863</v>
+      </c>
+      <c r="F16">
+        <v>0.39494013244711823</v>
+      </c>
+      <c r="G16">
+        <v>15.394940132447118</v>
+      </c>
+    </row>
+    <row r="17" spans="4:7">
+      <c r="D17">
+        <v>120</v>
+      </c>
+      <c r="E17">
+        <v>1.8732155679395459</v>
+      </c>
+      <c r="F17">
+        <v>0.14733515568501332</v>
+      </c>
+      <c r="G17">
+        <v>20.147335155685013</v>
       </c>
     </row>
   </sheetData>

</xml_diff>